<commit_message>
Updated current schedule and cleared previous dummy stats
</commit_message>
<xml_diff>
--- a/game-stats/Week2_WarBred_vs_Darkside.xlsx
+++ b/game-stats/Week2_WarBred_vs_Darkside.xlsx
@@ -527,7 +527,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -1313,7 +1313,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>OL/DL</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>OL/DL</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>OL/DL</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>OL/DL</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>OL/DL</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>OL/DL</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">

</xml_diff>